<commit_message>
feat: close chrome at finish process
</commit_message>
<xml_diff>
--- a/bots/MAGALU/links_afiliados_magalu.xlsx
+++ b/bots/MAGALU/links_afiliados_magalu.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2367,6 +2367,146 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>banheiro</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/banheira-de-bebe-kiddo-maresias-cinza/p/238454600/bb/ifba/</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/jdxxfv03</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:27:04</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>banheiro</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/banheira-para-bebe-dobravel-portatil-2-em-1-com-assento-45l-cinza-pipdip/p/da8ecg07f2/bb/ifba/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/te9ujmts</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:27:13</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>banheiro</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/cadeira-de-banho-higienica-d30-resistente-e-pratica-para-idoso-dellamed/p/ajd14134dh/cp/cbob/</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/w29xl1sf</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:27:35</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>banheiro</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/banheira-de-bebe-com-suporte-dobravel-maxi-baby-wish-branca-40l/p/240688100/bb/ifba/</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/th23l0l6</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:27:44</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: multiple keywords and loop
</commit_message>
<xml_diff>
--- a/bots/MAGALU/links_afiliados_magalu.xlsx
+++ b/bots/MAGALU/links_afiliados_magalu.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2507,6 +2507,726 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>hamburguer</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/modelador-de-hamburguer-maquina-industrial-2-discos-lcg-eletro/p/df0h9410f6/ud/mdlh/</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/8qmggcu9</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:53:25</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>hamburguer</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/prensa-molde-para-hamburguer-carne-forma-de-hamburguer-generico/p/fgf70adgd2/am/mods/</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/4c2nxx2r</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:53:36</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>hamburguer</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>3</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/modelador-de-hamburguer-artesanal-prensa-aluminio-bazar-do-saara/p/kc7ffb0a59/ud/mdlh/</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/wpn8cgvz</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:53:45</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>hamburguer</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>4</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/forma-modeladora-para-fazer-molde-hamburguer-manual-recheado-plasutil/p/dk3135jg43/ud/mdlh/</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/wgdd686u</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:53:53</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>hamburguer</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/modelador-de-hamburguer-artesanal-aro-12cm-aluminio-redar/p/hj65k8b861/ud/comp/</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/rbth70os</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:54:00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>hamburguer</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>6</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/forma-modelador-de-hamburguer-artesanal-caseiro-molde-para-hamburguer-gourmet-utensilios-cozinha-h-m/p/fj7ka0c476/ud/mdlh/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:54:23</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Não foi possível obter o link de afiliado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-de-mesa-britania-1500w-de-potencia-bcq10a/p/240305900/fj/celt/</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/uj7jfxlp</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:54:45</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-portatil-2000w-mondial-grand-steak-e-grill-ch-05/p/236675000/fj/chua/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:55:06</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Não foi possível obter o link de afiliado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-carvao-movel-california-preta-grelha-e-espetos-mor/p/ghd2j611ej/fj/chcv/</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/zlarvyj6</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:55:15</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>4</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-a-bafo-pequena-com-alta-eficiencia-no-preparo-de-carnes-e-grelhados-star-produtos/p/jh5a5g7df2/fj/chua/</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/j2x80d6f</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:55:24</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-britania-1500w-bcq40/p/238193400/fj/chua/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:55:47</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Não foi possível obter o link de afiliado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>6</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-montana-mor-03005/p/jaf13a1j94/fj/chcv/</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/z2gp44ib</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:55:57</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>7</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-movel-com-tampa-bafinho-45x35x32cm-tambor-mini-preta-hn/p/ef3hhk049f/fj/chcv/</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/ugpdkpdz</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:06</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>8</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-portatil-apartamento-sem-fumaca-grill-2000w-grande-linha-premium-bak/p/dj6bfhj8h1/fj/chua/</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/ic7er56s</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:13</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>9</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-portatil-apartamento-sem-fumaca-grill-2000w-grande-linha-premium-home-imports/p/hgfgfaj2c6/fj/chua/</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/k58sfrsa</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:22</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>10</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-grill-galvanizada-c-grelha-portatil-aco-anti-corte-kvell/p/kb9b8cjf14/fj/chua/</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/zt0ys40x</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:31</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>11</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-2000w-para-churrasco-110v-compacta-com-termostato-grelha-ajustavel-nza/p/af6f8k966k/fj/celt/</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/8s1kxj7b</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:40</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>12</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-movel-portatil-a-carvao-com-rodinhas-pro-tork-preto-grill-machine/p/gc009f997g/fj/chua/</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/vbp51077</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:49</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>13</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-portatil-2000w-mondial-grand-steak-e-grill-ii-ch-06/p/236675200/fj/chua/</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/dz11rmkn</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:56:57</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>14</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-110v-1500w-sem-fumaca-grelhador-de-mesa-portatil-churrasco-cozinha-5-nivel-bak/p/edj950jjac/fj/jdim/</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/baalaqbc</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:57:05</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>churrasqueira</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>15</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/churrasqueira-eletrica-mondial-pratic-steak-gril-ch-07/p/237288100/fj/celt/</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/r9fv1z1n</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>12/08/2026 13:57:18</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat add magalu user authenticator
</commit_message>
<xml_diff>
--- a/bots/MAGALU/links_afiliados_magalu.xlsx
+++ b/bots/MAGALU/links_afiliados_magalu.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,381 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>quarto</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/guarda-roupa-de-casal-6-portas-e-guarda-roupa-de-casal-lite-6-portas-para-quarto-grande-com-cabideiro-prateleiras-e-gavetas-cor-off-white-e-2-gavetas-maxi-do-brasil/p/ej891ba89k/mo/guro/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>R$ 899,90</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>quarto</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/quarto-de-bebe-completo-com-berco-comoda-e-guarda-roupa-henn-ternura-branco-e-jequitiba/p/238472900/mo/qdbc/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>R$ 2.849,90</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-sala-turim-para-tv-ate-65-polegadas-com-pes-madeira-moveis-bechara/p/bd54f5g74k/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/7r5wyofp</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ou R$ 367,83</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:02:32</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-sala-rubi-1-2-para-tv-ate-50-2-portas-pe-madeira-macica-moveis-bechara/p/feb36akh4g/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/l83rpea8</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ou R$ 316,00</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:02:47</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-para-sala-tv-ate-75-polegadas-2-portas-1-gaveta-reims-madesa/p/gjh61f407b/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/cqswnra3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>R$ 549,99</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ou R$ 431,99</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:02:58</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-sala-florenca-para-tv-ate-70-polegadas-com-pes-madeira-moveis-bechara/p/ghge305f23/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/m2oxm9xr</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ou R$ 459,79</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:03:14</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-bancada-sala-de-estar-para-tv-50-55-60-70-polegadas-sevilla-movelove-2-portas-1-gaveta-lukaliam-moveis/p/dkd57akc0d/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/evry4ftu</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ou R$ 478,63</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:03:31</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-sala-estar-tv-55-polegadas-madeira-white-organizador-deltre/p/bejf052e58/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/uo7gslz7</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>R$ 424,05</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ou R$ 352,74</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:03:44</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-para-sala-estar-malbec-wood-tv-ate-55-giga-moveis/p/kkf5ac5f1g/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/ewlj7a7c</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ou R$ 284,99</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:04:00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/rack-home-classic-decoracao-casa-apartamento-pequeno-sala-estar-quarto-tv-32-polegadas-2-portas-lojas-comprou-chegou/p/bhf9h539g9/mo/racm/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/r2pefg97</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>R$ 299,90</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ou R$ 218,37</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>19/08/2026 23:04:12</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>